<commit_message>
20220513-1659 generate BzPerformance SQL Commands.
</commit_message>
<xml_diff>
--- a/Data/EXCEL/Transfer/BzPerformance/2102-BzPerformance-20220510.xlsx
+++ b/Data/EXCEL/Transfer/BzPerformance/2102-BzPerformance-20220510.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\OneDrive\myStocksPGMs\V2.0\xls2xlsx\transfer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORKSPACES\myStocksPGMs\V2.0\xls2xlsx\transfer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D052DB22-D742-4744-9200-BC01E7E6388F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06950EFA-416C-4659-A897-A4E2127E58D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6615" yWindow="5985" windowWidth="24855" windowHeight="14895"/>
+    <workbookView xWindow="1725" yWindow="780" windowWidth="20190" windowHeight="11205"/>
   </bookViews>
   <sheets>
     <sheet name="2102-BzPerformance-20220510" sheetId="2" r:id="rId1"/>
@@ -110,7 +110,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -276,7 +276,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="新細明體"/>
-      <family val="1"/>
+      <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
@@ -310,14 +310,6 @@
       <color rgb="FFFF0000"/>
       <name val="新細明體"/>
       <family val="1"/>
-      <charset val="136"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="新細明體"/>
-      <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
@@ -856,7 +848,7 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -865,7 +857,7 @@
     <xf numFmtId="0" fontId="20" fillId="33" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -880,22 +872,22 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1256,14 +1248,14 @@
   <dimension ref="A1:U36"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="9.25" customWidth="1"/>
-    <col min="4" max="4" width="9.625" customWidth="1"/>
-    <col min="5" max="5" width="9.25" customWidth="1"/>
-    <col min="6" max="6" width="9.625" customWidth="1"/>
-    <col min="7" max="17" width="9.25" customWidth="1"/>
-    <col min="18" max="18" width="9.375" customWidth="1"/>
-    <col min="19" max="20" width="9.25" customWidth="1"/>
-    <col min="21" max="21" width="10" customWidth="1"/>
+    <col min="1" max="3" width="7.5" customWidth="1"/>
+    <col min="4" max="4" width="7.875" customWidth="1"/>
+    <col min="5" max="5" width="7.5" customWidth="1"/>
+    <col min="6" max="6" width="7.875" customWidth="1"/>
+    <col min="7" max="17" width="7.5" customWidth="1"/>
+    <col min="18" max="18" width="7.625" customWidth="1"/>
+    <col min="19" max="20" width="7.5" customWidth="1"/>
+    <col min="21" max="21" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
@@ -3575,7 +3567,7 @@
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
   </mergeCells>
-  <phoneticPr fontId="25" type="noConversion"/>
+  <phoneticPr fontId="24" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>